<commit_message>
Add SUBS-011 to SUBS-020 to Subsidence Case Database — Batch 2 complete
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Subsidence_Case_Database.xlsx
+++ b/knowledge/case-databases/Subsidence_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1653,6 +1653,1056 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="120" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>DRN2951368</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Covea Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>30 Oct 2020</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — subsidence claim; inadequate investigation in 2010 (superficial inspection only) led to Covea applying the £15,000 excess introduced in 2011 rather than the £1,000 excess applicable in 2010; consumer argues the 2017 tree-root subsidence is a continuation of the 2010 claim</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Tree root-induced clay soil shrinkage at front of property; relationship between weather conditions and tree roots caused cyclical cracking that first manifested before 2010; tree removed and movement stabilised after 2017 investigation</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Covea: three distinct claims from three causes (1998, 2010, 2017); 2017 claim is subject to the £15,000 excess in force at that time; loss adjuster C found only differential movement in 2010 that was not worsening; tree implicated only from hot summer 2016 — a new event; CUE should record three claims</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Consumer: C's inspection in 2010 was superficial (three-day turnaround, no in-depth investigation); C subsequently said tree impact on 2010 cracks could not be ruled out; prior experts had recommended monitoring. Covea: original underpinning repairs (2002/3) remained in good order; C found differential movement in 2010 within the excess; 2017 investigation found tree impact from 2016 hot summer; three separate causes. FOS: prior history and experts' recommendations warranted more than a superficial investigation in 2010; C acknowledged tree impact on 2010 cracks could not be ruled out; tree root clay shrinkage is cyclical and weather-dependent — absence of worsening in one period does not confirm absence of cause; Covea has not shown on balance that 2010 cracks were unrelated to the tree; likely continuation from 2010; finely balanced but £1,000 excess is fair</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Record the 2017 claim as commencing in 2010; amend the CUE database to record two subsidence claims not three; apply the £1,000 excess applicable in 2010 (future claims remain subject to the current excess)</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Where a loss adjuster's inadequate investigation of an earlier claim prejudices the excess the consumer pays on a later related claim, FOS may direct the later claim be treated as a continuation of the earlier and apply the earlier excess; insurer duty under ICOBS to handle claims promptly and fairly, not unreasonably reject; tree root clay shrinkage is cyclical — weather-driven fluctuations in visible movement do not break the causal chain; insurer bears the burden of demonstrating that the later damage is a distinct new event to justify the higher excess applicable at the time of the later claim; CUE database must accurately reflect the number of distinct claims</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>Detailed investigation reports from the 2010 claim (none produced — C completed only a superficial inspection with no exploratory investigation within three days of attendance)</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>Property had prior subsidence history and experts had recommended further monitoring; Covea chose a new loss adjuster specifically to avoid thorough investigation; C's 2010 inspection was superficial — no in-depth investigation despite that history; C subsequently acknowledged tree impact on 2010 cracks could not be ruled out; tree root clay shrinkage is cyclical — not a constant; Covea has not shown on balance that 2010 cracks were unrelated to the tree; likely continuation from 2010 given original underpinning repairs (2002/3) remained in good order; finely balanced but fair outcome is £1,000 excess and two CUE entries</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>Loss adjusters instructed on a property with prior subsidence history must carry out a thorough investigation — a superficial visit that produces a final determination within three days is likely to be found inadequate by FOS; where an inadequate investigation in an earlier claim later prejudices the excess payable on a continuation claim, FOS will direct the higher excess to be replaced by the lower one applicable at the time of the earlier claim; tree root clay shrinkage claims are inherently cyclical — variation in movement between dry and wet years does not establish a new distinct event; insurer must demonstrate on balance that later damage is a new and distinct event before applying the higher current-period excess</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>IF inadequate_investigation_of_prior_claim AND later_damage_likely_related_by_same_cause THEN insurer_may_be_directed_to_treat_later_claim_as_continuation_applying_earlier_excess; IF property_has_prior_subsidence_history AND experts_recommended_further_investigation THEN superficial_inspection_is_inadequate; tree_root_clay_shrinkage_is_cyclical_so_absence_of_worsening_in_one_period_does_not_confirm_absence_of_cause; insurer_must_demonstrate_on_balance_that_later_damage_is_distinct_new_event_to_apply_higher_excess_applicable_at_later_date</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>DRN2951368.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-012</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3258437</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Red Sands Insurance Company (Europe) Limited</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>2 Jun 2022</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance — subsidence claim made in 2020 (same year as inception); Red Sands removed subsidence cover and declined claim on grounds that Mr P could not produce the specific certificate of adequacy or chartered surveyor's report required by the policy question, and therefore made a misrepresentation under CIDRA 2012</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Subsidence (cause and extent not concluded — loss adjuster had suggested monitoring before claim was declined when subsidence cover was removed; investigation incomplete)</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Red Sands: Mr P selected 'am able to provide' certificate of adequacy or chartered surveyor's report but could not produce either specific document; Red Sands would not have offered subsidence cover without those documents; Mr P should know more than a layman given his experience buying a property with prior subsidence history; damage may be linked to previous problems</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Mr P: openly disclosed prior subsidence history; believed his available evidence (confirmed accepted claim, loss adjuster explanation, drainage work completion, 2014 RICS mortgage valuation showing no structural movement) fulfilled the requirement; answered to best of knowledge as a layman. Red Sands: specific documentation required to manage risk; consumer could have used email or chat to clarify; consumer's experience of buying a subsidence-history property elevates his knowledge beyond layman level. FOS: CIDRA test is reasonable care not to misrepresent, not strict correctness; Mr P's evidence achieves broadly the same purpose as a certificate of adequacy — shows prior problem was dealt with normally; RICS mortgage valuation finding no structural movement goes further than a certificate would; buying a property with prior subsidence history does not import professional knowledge of subsidence or insurance; Red Sands is not disadvantaged by absence of a certificate format</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Red Sands to reinstate subsidence cover; consider the claim subject to policy terms and conditions (claim requires further investigation and monitoring before outcome can be determined)</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>CIDRA 2012 — test is reasonable care not to misrepresent, not strict correctness; where consumer's evidence achieves the same substantive purpose as specifically requested documentation (certificate of adequacy), insurer is not disadvantaged by absence of exact format and cannot establish a qualifying misrepresentation; RICS mortgage valuation finding no structural movement may provide broader reassurance than a certificate of adequacy; purchasing a property with a subsidence history does not import professional knowledge of buildings, subsidence or insurance claims — consumer remains a layman unless specific expertise is demonstrated</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>Certificate of adequacy from original insurer (not obtained); chartered surveyor's structural report (not obtained); conclusion on whether 2020 damage is linked to prior subsidence (monitoring required — investigation was abandoned when cover was removed)</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>CIDRA test is reasonable care; Mr P's documents show prior subsidence claim accepted by an insurer, cause identified (leaking drains), drainage work completed, RICS survey found no structural movement — this substantially achieves the purpose of a certificate of adequacy; Red Sands no more disadvantaged than if a certificate had been provided; Mr P is a layman — buying a house with subsidence history does not make him more expert in subsidence or insurance; not satisfied he failed his CIDRA duty; Red Sands has no CIDRA remedy; claim must be properly investigated</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>When relying on CIDRA to remove subsidence cover, insurer must show the consumer's answer failed to meet the 'reasonable care' standard — mere technical non-compliance with a document format requirement is insufficient; where the consumer's available evidence achieves the same substantive purpose as the specific document requested, the CIDRA test is met even if that exact format is absent; consumer's occupational or life experience importing relevant expertise must be specifically demonstrated — the fact of buying a property with subsidence history alone does not elevate the consumer above layman status; when removing cover and declining a claim simultaneously, the claim investigation should not be abandoned — FOS may require both steps to be undone</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>IF consumer_evidence_achieves_same_purpose_as_requested_document THEN CIDRA_reasonable_care_test_met_even_if_exact_format_absent; IF consumer_purchased_property_with_prior_subsidence_history THEN consumer_remains_layman_unless_specific_professional_expertise_demonstrated; IF insurer_removes_cover_under_CIDRA AND claim_investigation_incomplete THEN insurer_directed_to_reinstate_cover_and_complete_investigation; CIDRA_test_is_reasonable_care_not_strict_correctness</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3258437.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3387540</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Accredited Insurance (Europe) Limited</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>17 May 2022</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — new cracks noticed in 2020 (year of policy inception); AIL declined claim for pre-existing/maintenance-related damage exclusion; separately argued claim cost below £2,500 excess; also failed to renew policy after declining claim, leaving consumer without subsidence cover</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Subsidence caused by trees (AIL identified as cause after inspection; tree investigation and crack monitoring recommended before claim was declined)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>AIL: (1) damage pre-existing or maintenance-related — homebuyer's survey noted property needed repair and prior subsidence had occurred; policy excludes pre-inception events; (2) schedule of works £1,900 is below £2,500 subsidence excess</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Mr P: discovered new cracks August 2020; prior subsidence (approx 10 years earlier) was repaired by insurer; homebuyer's survey found no significant structural defects, no active movement. AIL: homebuyer's survey noted prior subsidence; inspection showed internal cracks (photos not annotated). FOS: excess argument — total claim value includes investigation and monitoring costs (likely &gt;£600) plus repair costs (£1,900) so overall value likely exceeds £2,500 excess; pre-existing exclusion — AIL's own inspection report did not comment on when subsidence started; homebuyer's survey found no active movement; no expert evidence that current subsidence pre-existed the January 2020 inception; burden of proof on AIL as party relying on exclusion; AIL failed to renew after declining claim — obligation to continue cover after accepted claim applies; wrongful denial effectively deprived consumer of subsidence cover at renewals 2021 and 2022</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Accept the subsidence claim; offer cover including subsidence from next renewal and confirm subsidence cover from January 2021 to January 2023; pay the difference between what Mr P paid for alternative cover and what he would have paid remaining with AIL; pay £500 compensation; consider consumer's professional costs (legal, arboricultural, tree surgery) incurred progressing claim after wrongful decline — confirm which are refunded or offset against excess</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Pre-existing damage exclusion — burden of proof on insurer relying on exclusion to show damage existed before inception; homebuyer's survey finding no active movement is strong evidence against pre-inception subsidence; excess applies to total claim value including investigation and monitoring costs, not just repair cost alone; insurer obliged to continue offering subsidence cover at renewal after accepting a claim; wrongful claim denial that leads to consumer losing subsidence cover at subsequent renewals creates liability for increased premium costs consumer paid to alternative insurers; consumer professional costs (surveyor, arboricultural, tree surgery) incurred in progressing a claim after wrongful denial may be refunded or offset against the excess</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>Expert opinion on when current subsidence began relative to policy inception; AIL inspection report timing commentary (not provided); confirmation of tree investigation and monitoring cost to establish whether excess was actually exceeded</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>Excess argument fails — total claim value includes tree investigation and crack monitoring (&gt;£600) plus £1,900 repair costs, likely exceeding £2,500; pre-existing exclusion fails — AIL's inspection did not state when subsidence started; homebuyer's survey found no active movement; no expert evidence of pre-inception subsidence; burden on AIL not discharged; AIL obliged to continue cover after accepted claim; failure to renew created obligation to pay increased premium costs consumer incurred</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>Insurer relying on a pre-existing damage exclusion must obtain and produce expert evidence that the current subsidence began before policy inception — it is not sufficient to note that prior subsidence occurred years earlier and was repaired; excess must be calculated against total claim value including all investigation, monitoring, tree works and repair costs — it is not limited to the repair schedule alone; insurer that wrongly declines a claim and then fails to renew the policy creates a compounded liability: the claim itself plus the increased premium costs the consumer paid elsewhere and the loss of subsidence cover for those renewal years</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>IF pre_existing_damage_exclusion_relied_upon THEN insurer_must_produce_expert_evidence_that_subsidence_existed_before_inception; IF homebuyer_survey_found_no_active_movement THEN strong_evidence_against_pre_inception_subsidence; excess_must_be_calculated_against_total_claim_value_including_investigation_monitoring_and_tree_costs; IF insurer_wrongly_declines_claim AND fails_to_renew THEN liable_for_claim_plus_increased_premium_costs_at_alternative_insurers; consumer_professional_costs_after_wrongful_decline_may_be_offset_against_excess_or_refunded</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3387540.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-014</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3427348</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Amtrust Europe Limited</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>9 May 2022</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Commercial landlord buildings insurance — cracking reported June 2021; Amtrust concluded longstanding movement from street view images (2012+) and 2008 pre-purchase survey; backdated removal of subsidence cover to 2017 (claiming misrepresentation at renewal) and declined claim on grounds movement is settlement not subsidence</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Longstanding differential settlement caused by different foundation depths between front and rear of building (front founded higher due to cellar construction; different depths cause very gradual differential downward movement); trees, drain leakage and clay shrinkage all ruled out by Amtrust specialists</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Residential let property (landlord/commercial policy — Insurance Act 2015 applies)</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Amtrust: (1) longstanding cracking and movement not disclosed at 2017 renewal when asked whether property had experienced stepped/diagonal cracking, subsidence, ground heave, landslip, movement or underpinning — answered 'No'; would not have provided subsidence cover if known; backdated subsidence cover removal to 2017. (2) Movement is settlement (differential foundation depths) not subsidence — settlement excluded under policy</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Mrs G: unaware of cracks as property was tenanted; disputes cracks were present; Amtrust's agents behaved badly during inspection. Amtrust: street view images from 2012 clearly show cracks; 2008 pre-purchase survey noted longstanding movement; landlord has responsibility to inspect and maintain; underwriting guide supports removing subsidence cover. FOS provisional: Mrs G misrepresented (should have answered 'Yes'); Insurance Act 2015 applies; BUT Amtrust's underwriting guide only removes subsidence cover for previous/existing confirmed subsidence — not for settlement or general movement; movement confirmed as settlement not subsidence; Amtrust did not demonstrate qualifying breach justifying subsidence cover removal under IA 2015. FOS final: Amtrust's oral argument that underwriters interpret guide more broadly than its text is insufficient — guide must demonstrate what Amtrust would have done; qualifying breach for subsidence cover removal not established; backdating unfair; claim decline for settlement is correct</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Amtrust to reinstate subsidence cover backdated to 2017; claim decline upheld — damage caused by settlement which is excluded under the policy</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Insurance Act 2015 (commercial landlord policy) — insurer must demonstrate a qualifying breach to apply a remedy; insurer's underwriting guide must specifically support the action taken; if underwriting guide only removes subsidence cover for confirmed previous/existing subsidence, insurer cannot extend that to settlement or general movement/cracking — it must show qualifying breach for the specific scenario; settlement and subsidence are distinct and separately addressed perils — insurer must apply the correct exclusion for the correct peril; misrepresentation on a broad question (including cracking/movement) does not automatically create a qualifying breach justifying removal of subsidence cover if underwriting criteria do not specifically address that scenario</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Amtrust underwriting guide provisions specifically addressing what the insurer would do if informed of cracking/movement that is not confirmed subsidence (guide only addressed confirmed subsidence explicitly); whether Mrs G received any communication about cracks from tenants</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Mrs G misrepresented — street view images from 2012 show longstanding cracks; should have answered 'Yes' at 2017 renewal; Insurance Act 2015 applies; qualifying breach requires showing what Amtrust would have done — underwriting guide only covers confirmed previous/existing subsidence; damage confirmed as settlement (different foundation depths) not subsidence; policy already excludes settlement as standard, so removing subsidence cover specifically would not have changed outcome for settlement damage; Amtrust hasn't demonstrated qualifying breach to support backdated removal of subsidence cover; backdating unfair; claim decline for settlement is fair and correct</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>Commercial landlord insurers relying on Insurance Act 2015 to backdate removal of subsidence cover must produce underwriting guide provisions specifically covering the disclosed risk scenario — a guide that only addresses confirmed subsidence does not justify removal of cover where the disclosed issue is settlement, cracking or movement; settlement and subsidence must be distinguished at claim stage — settlement is typically excluded as standard while subsidence requires specific cover; where a broad disclosure question captures general cracking/movement that turns out to be settlement (not subsidence), and the policy already excludes settlement, removing subsidence cover in addition is disproportionate and unsupported by standard underwriting criteria; landlord-policy misrepresentation cases under IA 2015 require specific demonstration that the remedy taken matches what the underwriting guide actually says</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>IF insurance_act_2015_applies AND insurer_claims_qualifying_breach THEN underwriting_guide_must_specifically_support_action_taken; IF underwriting_guide_addresses_only_confirmed_subsidence THEN it_does_not_support_removal_of_cover_for_settlement_or_general_cracking; settlement_and_subsidence_are_distinct_perils_requiring_separate_exclusion_analysis; IF movement_confirmed_as_settlement_not_subsidence THEN settlement_exclusion_applies_and_claim_decline_is_fair; misrepresentation_on_broad_movement_question_does_not_automatically_justify_removal_of_subsidence_cover</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3427348.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="120" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3581769</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Fairmead Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>3 Aug 2022</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — subsidence claim accepted (porch sinking, January 2020); dispute about whether drain repairs caused by the subsidence should be covered under one subsidence claim or a separate accidental damage claim with a separate £200 excess; also unresolved subsidence structural repairs and inadequate communication throughout</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Ground subsidence causing porch to sink; drains within area of influence damaged by subsidence movement; separate drain defects outside area of influence unrelated to subsidence; patio damage attributed to settlement not subsidence</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Fairmead: drain repairs within the area of subsidence influence covered under subsidence claim; drain repairs outside the area of influence not connected to subsidence — separate accidental damage claim with separate £200 excess; patio damage = settlement (not covered); faulty drainage design and missing lintels = defects in design/workmanship (not covered)</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Mr and Mrs C: all drain repairs and all damage on three sides should be covered under one subsidence claim. Fairmead: drains within influence area covered under subsidence; drains outside influence area dealt with separately. FOS: internal notes, loss adjuster breakdown and two receipts for £200 excess confirm a separate £200 excess was charged for drain repairs that were actually connected to and caused by the subsidence — despite Fairmead's assertion to the contrary; drain damage caused by and contributing to subsidence must be included under the one subsidence claim with the one subsidence excess; drain repairs outside the area of influence and genuinely unrelated to subsidence can legitimately be a separate claim; consumer-funded private repairs without expert evidence linking them to subsidence: not reimbursable; faulty design/workmanship and missing lintels not covered; further site investigation needed to confirm drain repairs are lasting and effective</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Carry out further investigation to confirm drain repairs under subsidence claim are lasting and effective; complete lasting and effective repair if not; investigate slabs near kitchen for subsidence damage and relay if confirmed; refund £200 accidental damage excess paid April 2020 with 8% simple interest from date of payment to settlement; update all internal and external records to reflect one subsidence claim; pay £500 compensation</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>Drain repairs caused by subsidence and contributing to it must be included under the subsidence claim with a single subsidence excess — insurer cannot split them into a separate accidental damage claim; drain repairs outside the area of subsidence influence that are genuinely unrelated to the movement may be treated as a separate claim; excess applies only once per subsidence event — insurer charging a second excess for subsidence-related drain repairs is incorrect; insurer must maintain accurate internal and external records — if records show two separate claims for the same subsidence event, they must be corrected; insurer must be given first opportunity to investigate and rectify its own repairs before consumer can demand independent survey</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>Expert evidence demonstrating the privately-funded drain repairs (outside area of influence) were caused by or contributed to the subsidence; confirmation of whether slabs outside kitchen moved due to subsidence</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>Internal notes, loss adjuster breakdown and consumer receipts all confirm a separate £200 accidental damage excess was charged for drain repairs actually related to subsidence — this contradicts Fairmead's assertion that all was handled under one claim; the fair principle is that subsidence-related drain repairs belong under one subsidence claim with one excess; Fairmead's stated policy on this point (apply one subsidence claim for subsidence-related drains) was not followed in practice; further drain investigation needed as repairs may be defective; slabs to be reviewed at same time; communication was poor throughout; £500 compensation appropriate</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>When drain repairs are split between 'subsidence-related' and 'unrelated', the insurer must correctly categorise each part and charge only one excess for all subsidence-related elements — charging a separate accidental damage excess on drain repairs within the area of influence is incorrect and will be reversed; internal claim records must accurately reflect what was covered and how — inconsistency between notes and practice creates both a rectification obligation and a compensation liability; insurer must be given first opportunity to inspect and rectify its own repair work before consumer-requested independent surveys are authorised</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>drain_repairs_caused_by_subsidence_and_contributing_to_it_must_be_included_under_subsidence_claim_with_single_excess; IF insurer_charges_separate_accidental_damage_excess_for_drain_repairs_within_subsidence_area_of_influence THEN excess_must_be_refunded; drain_repairs_outside_area_of_influence_and_genuinely_unrelated_may_be_separate_claim; IF consumer_alleges_insurer_repairs_defective THEN insurer_must_reinvestigate_before_independent_survey_is_directed; insurer_records_must_accurately_reflect_one_subsidence_claim_for_one_subsidence_event</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3581769.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-016</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3682901</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>7 Oct 2022</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance — subsidence accepted (November 2020); insurer identified defective drains as the cause but refused to fund drain repairs under the subsidence claim, citing the accidental damage section's 'sudden' requirement; told consumers to arrange and fund drain repairs themselves before the subsidence claim could progress</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Ground movement caused by defective drains (leaking or washing away supporting ground); drain defects occurred gradually over time — not sudden; drain repair is required before the structural subsidence repairs can be carried out to prevent recurrence</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's: drain defects fall under the accidental damage section of the policy; the accidental damage section requires a sudden event and drain defects occurred gradually; accidental damage section therefore does not apply; consumers must fund and arrange drain repairs themselves before insurer will progress subsidence repairs</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's: separate accidental damage section covers drains; 'sudden' requirement not met. FOS: insurer's obligation to carry out a lasting and effective repair when a valid subsidence claim is accepted extends beyond the literal scope of the policy — it includes repairing the underlying cause of the subsidence to prevent recurrence; drain repair is required for a lasting and effective repair; whether the drains are separately covered under the accidental damage section is irrelevant — they must be repaired under the subsidence section to fulfil the lasting and effective repair obligation; analogous to underpinning (which no insurer disputes); one excess only; Mr and Mrs F are in their 90s and paid from savings — aggravating factor for compensation</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Reimburse Mr and Mrs F for cost of drain repairs on receipt of evidence of costs; pay 8% simple interest per annum from date of payment to settlement; charge only one excess for the entire claim; deal with all repairs as one subsidence claim; pay £300 total compensation (£150 additional)</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Insurer's duty to carry out a lasting and effective repair under an accepted subsidence claim extends to repairing the underlying cause of the subsidence (e.g. defective drains) even if that cause is not explicitly covered under the policy's accidental damage section; where drain repair is required before structural repairs can be durable, the insurer must fund it as part of the subsidence claim regardless of whether the 'sudden' requirement in the accidental damage section is met; this obligation is analogous to underpinning — it is a necessary precondition for an effective repair; only one excess applies to one subsidence event; consumer vulnerability (advanced age, using savings) is a relevant factor in setting compensation level</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>N/A — the factual situation was not in dispute; Lloyd's accepted the drains needed repair but disputed who should pay</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's accepted subsidence and obligation to repair; lasting and effective repair requires removal of the underlying cause; drain repair is required to prevent subsidence recurring — without it, structural repairs will fail; whether drains are covered under the accidental damage section is irrelevant; insurer's obligation under the subsidence section overrides the separate section analysis; analogous to underpinning, which all insurers acknowledge as their obligation; one excess for one event; Mr and Mrs F are in their 90s and paid from savings — this aggravates the D&amp;I impact and justifies £300 total compensation</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>When a subsidence investigation identifies defective drains as the root cause, the insurer must fund those drain repairs as part of the subsidence claim even if the policy's accidental damage section does not technically cover the drain defect — the lasting and effective repair obligation overrides the section-by-section analysis; an insurer cannot use an accidental damage 'sudden event' requirement to avoid funding drain repairs that are the identified cause of an accepted subsidence claim; one excess applies per subsidence event — a second excess for the drain element is incorrect; consumer age and financial vulnerability are relevant to D&amp;I compensation quantum</t>
+        </is>
+      </c>
+      <c r="T17" s="5" t="inlineStr">
+        <is>
+          <t>IF defective_drains_are_identified_cause_of_accepted_subsidence THEN insurer_must_fund_drain_repairs_under_subsidence_claim; drain_repair_required_for_lasting_and_effective_repair_must_be_funded_regardless_of_accidental_damage_section_limitations; IF drain_defects_occurred_gradually_and_accidental_damage_section_requires_sudden_event THEN insurer_cannot_use_that_to_avoid_drain_repair_obligation_under_subsidence_section; one_excess_applies_per_subsidence_event; consumer_vulnerability_and_age_are_relevant_factors_in_compensation_quantum</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3682901.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3929594</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>24 Jul 2023</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — complaint about premium and subsidence excess increases at April 2021 and April 2022 renewals following accepted subsidence claim (November 2020 claim accepted; second claim recorded March 2022); AXA failed to respond to complaint</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Subsidence (cause not specified — first claim accepted and cash settled November 2022; second claim recorded March 2022 and under investigation)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>AXA: subsidence excess increases based on underwriting criteria and claim reserve (amounts spent and expected to be spent on claim) at each renewal; premium increases correctly calculated per AXA's underwriting model; second claim at 2022 renewal further increased risk</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Mr and Mrs I: increases unfair. AXA: detailed premium calculations submitted; excess based on claim reserve; individual underwriter would not have calculated differently. FOS investigator: premium increases correct; excess increase not justified at the level set. AXA: provided further underwriting comments challenging investigator. FOS ombudsman: ABI guidance requires renewal terms to be reasonable not merely technically correct per underwriting formula; premium increases are both correct and reasonable given subsidence claim history and second claim at 2022 renewal; excess — AXA set it at £10,000 based on an overstated reserve; applying AXA's own criteria to actual accurate claim values, £5,000 was the appropriate excess at both 2021 and 2022 renewals; both parties accepted £5,000 figure</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>AXA to reduce the subsidence excess at the 2021 and 2022 renewals to £5,000</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>ABI guidance on continuation of cover after subsidence claim requires insurer to offer renewal on reasonable terms — reasonableness is the standard, not merely mathematical accuracy of the underwriting formula; premium increases post-subsidence claim are justified if correctly calculated per the insurer's underwriting criteria AND not unreasonable; subsidence excess post-claim must reflect the actual claim value (reserve), not an inflated or over-estimated amount — FOS will review against both the insurer's own criteria and the accuracy of the reserve figures used; a second subsidence claim provides additional justification for a premium increase at that renewal</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Accurate claim reserve at each renewal (AXA used overstated reserve to calculate excess — FOS applied actual settled values to determine £5,000 appropriate)</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>Premium increases correctly calculated per AXA criteria and reasonable given subsidence history and second claim; excess incorrectly set at £10,000 — based on overstated reserve figures; applying AXA's own underwriting criteria to accurate claim values, £5,000 is the fair excess at both renewals; ABI standard requires reasonable terms, not just formula compliance; second claim at 2022 renewal legitimately contributed to premium increase; AXA did not respond to the original complaint — a separate failing acknowledged</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>Post-subsidence claim excess setting must use accurate claim reserve values — using an overstated reserve to set a higher excess will be corrected by FOS to the level the insurer's own criteria would produce when applied to actual values; premium increases must satisfy the ABI reasonableness standard, not just the insurer's internal pricing model; when a second subsidence claim is recorded, it provides a stronger basis for renewal excess and premium adjustments; insurer failure to respond to a complaint on time is a separate service failing but does not override the substantive analysis of whether the pricing was fair</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>subsidence_excess_at_renewal_must_be_calculated_on_accurate_claim_reserve_not_overstated_estimate; IF insurer_excess_based_on_overstated_reserve THEN FOS_will_reduce_excess_to_level_justified_by_actual_claim_values_under_insurers_own_criteria; ABI_continuation_guidance_requires_renewal_terms_to_be_reasonable_not_merely_formula_correct; second_subsidence_claim_provides_additional_basis_for_excess_and_premium_increase_at_that_renewal</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3929594.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-018</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4190935</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>15 Jan 2024</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance — Society of Lloyd's underwriter (U) withdrew from the home insurance market; Mr M had an open subsidence claim from March 2020; underwriter provided a 3-month extension then a 12-month renewal with £10,000 excess, but did not renew at expiry (August 2021); broker could not find replacement cover with subsidence; ABI guidance on continuation of cover not followed</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Subsidence (cause not specified — claim accepted in 2020; investigation ongoing when cover was removed)</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's / underwriter U: commercial decision to withdraw from providing the policy type Mr M held; decision applied to all policyholders with that policy type, not just Mr M; U not obliged to provide insurance; broker was given adequate time to find alternative cover</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Mr M: cannot find subsidence cover elsewhere due to open claim; disadvantaged by market withdrawal. SoL: ABI guidance does not require insurers withdrawing from the market to make exceptions or find alternative cover for policyholders; withdrawal applied to all such policyholders not just Mr M; extension provided sufficient notice. FOS: ABI guidance applies regardless of ABI membership (industry good practice); guidance's block transfer provisions demonstrate its spirit — insurer ceasing to provide cover should arrange for policyholders not to be disadvantaged; if U had not withdrawn from the market, Mr M would have had continuing cover; U took no steps beyond a short extension to arrange alternative cover for Mr M; other insurers in similar positions have made exceptions, arranged policy transfers or subsidised specialist cover; inability to arrange alternative cover not actively demonstrated; not sufficient that continued cover is merely unwanted — must show it is impossible</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's to arrange for an underwriter (U or otherwise) to provide home insurance including subsidence cover to Mr M on reasonable terms, backdated to when his policy with U ended; premium and terms must not be set in a way that effectively prevents access to the ongoing subsidence cover</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>ABI guidance on continuation of cover following a subsidence claim applies to non-ABI members as a statement of industry good practice; the guidance applies even when an insurer withdraws from the home insurance market — withdrawal from the market is not listed as an exception; insurer withdrawing from the market must take reasonable steps to ensure the spirit of the guidance is achieved for policyholders with open/prior subsidence claims — this includes arranging alternative cover, subsidising specialist cover, or making an exception; the block transfer provisions of the guidance demonstrate the intent that stopping insurers must protect continuing-cover obligations; insurer preference not to provide cover is different from inability to provide cover — inability must be actively demonstrated; cover arranged for continuing-cover compliance must not be priced or structured so as to effectively prevent access</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Evidence that Society of Lloyd's or underwriter U actively attempted and failed to arrange alternative subsidence cover for Mr M (never pursued)</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>ABI guidance applies regardless of ABI membership; guidance applies to market withdrawal scenario — not listed as exception; block transfer provisions show guidance intends stopping insurers to arrange ongoing cover; if U had remained in market, Mr M would have had continuing cover — market withdrawal directly disadvantaged him; U provided short extension only and then left Mr M without subsidence cover; other insurers in similar situations found solutions (exceptions, transfers, subsidised specialist cover); SoL asserted alternative impossible but never actively explored it; not persuaded that arranging cover is impossible; SoL must arrange cover — it does not need to set up the policy itself, only to arrange an underwriter to provide it; terms must not effectively prevent access</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>An insurer withdrawing from the home insurance market must take proactive steps to protect policyholders with open or prior subsidence claims — the ABI continuation guidance is not disapplied by market exit; acceptable steps include making an exception for affected policyholders, arranging a block transfer to another insurer, or subsidising the difference between the existing premium and a specialist provider; merely telling the broker to find alternative cover and providing a short extension is insufficient; insurer must actively explore whether alternative arrangements are possible before asserting they cannot be made; any alternative cover arranged must be genuinely accessible — priced or structured so as to effectively prevent access is non-compliance</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>ABI_continuation_guidance_applies_to_non_ABI_members_as_industry_good_practice; ABI_continuation_guidance_applies_even_when_insurer_withdraws_from_home_insurance_market; IF insurer_withdraws_from_market AND policyholder_has_open_subsidence_claim THEN insurer_must_take_reasonable_steps_to_arrange_alternative_cover; acceptable_steps_include_exception_for_affected_customers_OR_block_transfer_OR_subsidy_for_specialist_cover; insurer_preference_not_to_provide_cover_is_not_the_same_as_inability_inability_must_be_demonstrated; alternative_cover_must_not_be_priced_so_as_to_effectively_prevent_access</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4190935.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4813489</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Kennett Insurance Brokers Limited</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>23 Apr 2025</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Buildings insurance — broker (Kennett) failed to declare Mr and Mrs D's 2003 subsidence claim when arranging new buildings insurance; insurer discovered discrepancy when a new subsidence claim was made in summer 2022 and avoided the policy; complaint against broker for omitting the prior claim from the application</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>2003 subsidence (cause not specified — handled by prior insurer); 2022 subsidence (investigation not completed — insurer avoided policy before investigation)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Kennett: standard wording requires consumers to verify accuracy of insurance documentation; Mr and Mrs D never flagged the omission over many years; Mr D was advised not to move away from the insurer who handled the 2003 claim but chose to do so; cannot establish exactly how the subsidence claim was removed from records</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Mr and Mrs D: trusted Kennett as longstanding broker (40+ years); Kennett knew about 2003 subsidence claim; should not need to audit broker's work annually. Kennett: cannot be certain how or when claim was removed from records; consumers had opportunity to review paperwork. FOS: likely Kennett's error caused the omission before the 2014 policy was taken out; demands and needs statements from 2017–2021 all referenced a subsidence excess, reasonably leading consumers to believe prior claim was properly declared; some policy schedules should have alerted them but not all required a claims history section; Kennett accepts it should have checked more closely when arranging policies; distress caused by Kennett's failure to maintain accurate records over a long relationship is clear; £150 compensation appropriate; insurer's avoidance handled in a separate complaint</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Kennett Insurance Brokers Limited to pay Mr and Mrs D £150 compensation for distress and inconvenience</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>Broker has a professional duty to accurately record and carry forward material claims history — including prior subsidence claims — when arranging insurance for longstanding clients; a broker who has knowledge of a prior subsidence claim and later arranges insurance that omits it is likely responsible for that omission; longstanding broker relationship and consumer trust do not transfer the broker's duty of care to the consumer; inclusion of a subsidence excess in renewal documents issued over multiple years can reasonably mislead a consumer into believing the prior claim is properly declared</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>Exact process and timing by which the 2003 subsidence claim was removed from Mr and Mrs D's insurance records (passage of time makes certainty impossible)</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>2003 subsidence not in dispute; Kennett knew about it; Kennett accepts omission occurred; likely Kennett's error before 2014; demands and needs statements consistently referenced subsidence excess, giving consumers reasonable comfort that the prior claim was properly declared; primary responsibility rests with Kennett; consumers could have been more vigilant but Kennett bears the main duty; insurer avoidance separately handled; £150 compensation appropriate for distress from a 40-year broker relationship ending in avoidance</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>Brokers placing insurance for clients with known prior subsidence claims must verify that each new policy application and subsequent renewals accurately reflect the subsidence claim history — repeated year-on-year omission cannot be blamed on the consumer; where a broker's own documents (demands and needs statements) reference a subsidence excess, consumers will reasonably but incorrectly believe the prior claim is properly declared — this reduces consumer contributory responsibility; insurer avoidance arising from broker omission creates both a broker compensation liability and a separate insurer-facing complaint</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>broker_must_accurately_record_prior_subsidence_claim_in_each_new_policy_application_it_arranges; IF broker_knew_of_prior_subsidence_claim AND arranged_policy_that_omitted_it THEN broker_is_likely_responsible_for_omission; IF renewal_documents_reference_subsidence_excess THEN consumer_reasonably_believed_prior_claim_was_declared; broker_omission_creating_insurer_avoidance_creates_broker_liability_for_D_and_I_and_separate_insurer_complaint</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4813489.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-020</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4883553</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>30 Sep 2024</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance — AXA removed subsidence, landslip and heave (SLH) cover entirely at the April 2023 renewal following two accepted subsidence claims (2020 and 2022); AXA cited risk appetite and claim history; SLH cover also absent from April 2024 renewal</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Subsidence (two accepted claims; specific causes not detailed in this decision — decision concerns cover removal, not cause investigation)</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>AXA: two subsidence claims increased risk beyond risk appetite; scenario not addressed by underwriting criteria so individual underwriter decided to remove SLH cover; entitled to refuse cover outside risk appetite; offered to 'consider' SLH in future</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Mrs I: purchased specialist non-standard insurance specifically covering subsidence; unfair to remove cover because she made claims against it; left in vulnerable position with subsidence history and no cover. AXA: two claims increased risk; happy to 'consider' SLH; underwriting criteria did not address multiple claims scenario. FOS investigator: AXA (ABI member) failed to act in line with ABI guidance; 'consider' is insufficient; recommended reinstatement backdated. FOS ombudsman: ABI guidance requires continuation of subsidence cover after a claim; guidance acknowledges problem cases (repeated subsidence, non-disclosure) but directs cover be provided wherever possible even in those cases; two subsidence claims is the scenario the guidance is specifically designed to address; it cannot be a compelling reason to remove cover; AXA must reinstate SLH for April 2023 and April 2024 renewals; vague offer to 'consider' is not an offer of cover</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>AXA to amend April 2023 and April 2024 policies to include subsidence, landslip and heave cover; pay £250 compensation</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>ABI guidance on continuation of cover — ABI member insurer that has dealt with a subsidence claim must normally continue to offer subsidence cover on the property; guidance explicitly acknowledges problem cases including repeated subsidence and requires cover to be provided wherever possible even in those cases; two subsidence claims cannot be a compelling reason to remove cover — they are the exact scenario the guidance is designed to remedy; insurer's 'risk appetite' is not a compelling reason that overrides ABI guidance obligations; offer to 'consider' providing SLH cover is not an offer of cover and does not satisfy the continuation obligation; only a risk fundamentally outside usual underwriting criteria (analogous to fraud) could justify departure from the continuation obligation</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>AXA's written underwriting criteria for scenarios involving two or more subsidence claims (decision was made by individual underwriter in absence of applicable criteria)</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>AXA is an ABI member — guidance binding; guidance requires continuation of SLH cover after subsidence claim; guidance recognises problem cases (repeated subsidence) and requires cover wherever possible even then; two claims is not a compelling reason to remove cover — it is the problem the guidance exists to address; AXA produced no compelling reason beyond two claims; AXA's 'consider' offer is insufficient — positive reinstatement required; April 2023 and 2024 policies must be amended; £250 compensation for unnecessary distress (related case DRN-3929594 had already reduced the excess to £5,000 at those same renewals)</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>ABI member insurers cannot rely on 'risk appetite' or 'claim history' as justification for removing SLH cover after multiple subsidence claims — the ABI continuation guidance specifically addresses repeated subsidence as a problem case and requires cover wherever possible; absence of underwriting criteria for a multiple-claim scenario means a commercial decision by an individual underwriter is not supported by written criteria and will be reviewed and overturned by FOS; the continuation obligation is not satisfied by an offer to 'consider' providing cover in future — it requires positive provision of cover; where a prior FOS decision has already corrected the excess for the same policy period, removal of SLH cover from the same renewal is an additional and independent breach of the ABI guidance</t>
+        </is>
+      </c>
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>ABI_member_insurer_must_continue_SLH_cover_after_subsidence_claim; two_subsidence_claims_are_not_a_compelling_reason_to_remove_cover_they_are_the_scenario_the_guidance_addresses; IF insurer_removes_SLH_cover_citing_risk_appetite_or_claims_history THEN removal_is_unfair_unless_compelling_reason_beyond_subsidence_itself_exists; offer_to_consider_cover_is_not_an_offer_of_cover; IF individual_underwriter_decision_not_supported_by_written_underwriting_criteria THEN decision_is_more_easily_overturned_by_FOS; departure_from_ABI_continuation_obligation_requires_compelling_reason_analogous_to_fraud_not_merely_commercial_unwillingness</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4883553.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add SUBS-021 to SUBS-030 to Subsidence Case Database — Batch 3 complete
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Subsidence_Case_Database.xlsx
+++ b/knowledge/case-databases/Subsidence_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2703,6 +2703,1056 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="120" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4950435</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>15 Apr 2025</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — outbuilding crack damage recorded and cash settled by AXA as subsidence without physical inspection (loss adjuster based decision solely on consumer's photos/videos); consumer's stonemason and chartered structural engineer both concluded damage was not subsidence; AXA agreed to reclassify record from subsidence to accidental damage but disputed reimbursing engineer's report cost and recalculating premiums</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Not subsidence — outbuilding cracking attributed to accidental damage; initial subsidence classification made without physical inspection or adequate investigation; chartered structural engineer confirmed no subsidence following detailed assessment</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Peril Classification Dispute</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>AXA: claim was properly recorded as subsidence based on photos/videos; loss adjuster's video call failed but assessment was adequate; consumer received benefit of settlement (repairs made from cash); engineer report cost not reimbursable as consumer had already benefited; premiums correctly calculated at time of renewal</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>AXA loss adjuster C: assessed via consumer's photos/videos only (video call failed; no physical inspection); brief summary report with no detailed rationale; recorded damage as subsidence. Miss B's stonemason: did not think damage caused by subsidence. Miss B's chartered structural engineer S (£696 report): physical inspection not possible (repairs done); detailed analysis of photos and other information; concluded damage was not subsidence and not covered by any policy peril. FOS: subsidence claims require physical inspection by appropriately qualified person — remote assessment from consumer photos only is inadequate; S's analysis was more persuasive and compelling than C's brief summary; weight of evidence firmly against subsidence as cause of damage</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>Reclassify claim record from subsidence to accidental damage internally and externally; recalculate 2023 and 2024 premiums with accidental damage classification and refund any overpayment plus 8% simple interest; reimburse £696 for S's engineering advice; pay £400 compensation for distress and inconvenience</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>Subsidence claims require physical inspection by an appropriately qualified person (chartered structural engineer, surveyor) — remote assessment based solely on consumer-provided photos/videos without physical inspection is inadequate and challengeable; incorrect subsidence recording causes lasting harm to premium costs and insurability that is independently compensable; where insurer's inadequate investigation causes consumer to commission independent engineering evidence, insurer must reimburse that cost; insurer that cash settles a non-covered claim as subsidence without adequate investigation cannot reclaim the settlement if consumer has spent funds on repairs; all premiums charged at a higher-risk (subsidence) rate must be reviewed and any overpayment refunded when the classification is corrected</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>C's detailed investigation rationale (only a brief summary was produced); physical inspection of damage before repairs were completed (not possible as repairs had already been carried out by the time claim was reconsidered)</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>Subsidence claims require a physically qualified inspection — C's assessment was based only on consumer's photos after a failed video call; C's report was brief with little explanation; S is a chartered structural engineer who provided detailed reasoning from available information; weight of evidence firmly against subsidence; AXA settled a non-covered claim without adequate investigation; Miss B had no realistic choice but to commission S's advice given AXA's inadequate investigation and failure to act on stonemason's concerns; AXA itself compounded its mistake by suggesting Miss B obtain engineering advice and then disputing the cost; no need to recover settlement as that was AXA's mistake and consumer used funds on outbuilding repairs; premiums must be recalculated</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>Initial subsidence classification made without physical inspection creates a risk that the claim is misrecorded with lasting consequences for the consumer (premium increases, difficulty obtaining insurance); once a consumer challenges a subsidence classification with professional evidence, insurer must genuinely review — failing to do so compels the consumer to incur further professional costs that become the insurer's liability; where a claim is wrongly recorded as subsidence without adequate investigation, insurer must correct the classification in all records and refund all consequential premium overpayments, but need not recover the original settlement payment if the consumer spent the funds on repairs</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>IF subsidence_classification_based_solely_on_consumer_photos_without_physical_inspection THEN investigation_is_inadequate_and_classification_is_challengeable; IF insurer_fails_to_act_on_consumer_challenge_to_subsidence_classification AND consumer_commissions_engineer_report THEN insurer_must_reimburse_engineer_costs; incorrect_subsidence_recording_must_be_corrected_internally_and_externally_in_all_systems; insurer_that_settles_uncovered_claim_as_subsidence_cannot_reclaim_settlement_if_consumer_spent_funds_on_repairs; IF claim_classification_corrected_from_subsidence_to_other_peril THEN all_premiums_at_higher_risk_rate_must_be_reviewed_and_overpayment_refunded</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4950435.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="120" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-022</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>DRN5217766</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>St Andrew's Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>2014 (est.)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance — conservatory subsidence claim (June 2011); two St Andrew's surveyors confirmed subsidence since 2003 but estimated repair cost below £1,100 excess; initial cause identified as clay shrinkage from neighbour's hedge; soil sample taken only after FOS complaint showed hedge roots were dead and soil not desiccated — initial cause hypothesis disproven; dispute about repair scope and adequacy of investigation</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Subsidence to conservatory on shallow foundations; initial cause (clay shrinkage from neighbour's hedge) disproven by soil analysis (roots dead, soil not desiccated); actual current cause undetermined at time of decision — requires proper investigation</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>St Andrew's: both surveyors confirmed subsidence since 2003; proposed limited repair scope (flashing, wall section, mastic fill) is adequate; estimated cost below £1,100 excess; historic settlement predates cover and St Andrew's not liable for demolish/rebuild; betterment principle limits liability for deeper foundations</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>St Andrew's surveyors: subsidence from hedge since 2003; limited repair scope adequate and cost below excess; deeper foundations would be betterment. St Andrew's surveyor (later, after soil sample): roots dead, soil not desiccated; cause may be shrinkage of made and deeper soils aggravated by vegetation — cause uncertain. Mrs A: conservatory continues to move; gap between conservatory and main house widening; contractors would not quote for proposed limited works as they said it would not solve the problem; 2000 valuation report showed no subsidence at time of purchase. FOS: soil sample arranged during FOS investigation (not proactively by St Andrew's) showed hedge was not the cause; St Andrew's surveyor acknowledged cause is now uncertain; without identifying cause, St Andrew's cannot confirm what scope of works is adequate or that repair cost is below the excess; insurer must carry out a proper investigation before asserting works are sufficient</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>St Andrew's Insurance Plc to carry out appropriate investigation to determine the cause of the current conservatory subsidence; then reassess what works need to be carried out to ensure an effective and lasting repair; pay Mrs A £500 compensation for distress and inconvenience from St Andrew's failure to properly investigate</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>Insurer must identify the cause of subsidence before determining the scope of repair works — without knowing the cause, it cannot establish what constitutes a lasting and effective repair or confirm repair cost is below the policy excess; where initial cause hypothesis is disproven by investigation, insurer must reinvestigate rather than defaulting to the original repair plan; obligation to carry out a lasting and effective repair may require demolish and rebuild if investigation shows it is necessary — betterment argument only limits what insurer funds for improvements beyond what is needed for an effective repair; argument that repair cost is below excess cannot be used to avoid investigation if the effectiveness of proposed repairs is uncertain; delay in investigating ongoing movement that consumer has repeatedly reported causes compensable distress</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>Root identification and soil desiccation data at time of 2011 inspection (soil sample only taken years later during FOS investigation, not arranged proactively); monitoring data to confirm whether conservatory movement is ongoing and its current rate</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Both St Andrew's surveyors confirmed subsidence since 2003; dispute was about scope of repair and cause; soil sample (arranged only after FOS complaint) showed hedge roots were dead and soil not desiccated — hedge was not the cause; St Andrew's own surveyor acknowledged this and conceded cause is uncertain; without knowing cause, St Andrew's cannot determine extent of liability or confirm proposed works are adequate; investigation could and should have been arranged years earlier; Mrs A witnessed continuing movement throughout; £500 appropriate for significant distress from failure to properly investigate over an extended period</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>Insurer investigating conservatory or structure subsidence must confirm the cause with adequate investigation before making any claim about repair scope or cost — assertions that repair cost is below excess are premature if cause is unknown; where cause investigation disproves initial field hypothesis (e.g. soil sample shows hedge roots dead and soil not desiccated), insurer must arrange further investigation proactively, not only when forced to do so by FOS complaint; consumer evidence of continuing movement must be taken seriously — if movement is ongoing and cause is unconfirmed, the insurer's obligation to carry out a lasting and effective repair is engaged and the excess argument cannot be relied upon</t>
+        </is>
+      </c>
+      <c r="T23" s="5" t="inlineStr">
+        <is>
+          <t>IF cause_of_subsidence_not_identified THEN insurer_cannot_determine_scope_of_repair_or_confirm_cost_is_below_excess; IF initial_cause_hypothesis_disproven_by_investigation THEN further_investigation_required_before_repair_scope_finalised; IF consumer_reports_ongoing_movement AND insurer_has_not_monitored THEN insurer_must_arrange_investigation_and_monitoring; delay_in_investigating_ongoing_movement_reported_by_consumer_causes_compensable_distress; excess_argument_cannot_be_relied_upon_when_cause_unknown_and_repair_effectiveness_is_uncertain</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>DRN5217766.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="120" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5220010</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>15 Jan 2025</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Landlord property insurance — garden/patio landslip caused by removal of adjacent retaining land by commercial construction; UKI's expert confirmed no subsidence to main building and identified cause as landslip; garden/patio damage excluded as yard; at 2023 renewal UKI removed subsidence cover citing underwriting criteria for properties showing signs of or suffering subsidence; consumer unable to obtain subsidence cover elsewhere</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Landslip and ground movement caused by removal of retaining land along shared boundary during commercial multi-storey building development; no subsidence to main building foundations identified; movement is downward slope from loss of lateral support, not clay shrinkage subsidence</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Residential let property (landlord insurance — Churchill/UKI)</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>UKI: (1) claim — main building undamaged; garden/patio damage excluded as yard under subsidence section of policy. (2) Cover removal — risk address showed signs of subsidence or had suffered subsidence per underwriting criteria; underwriting team confirmed subsidence cover could not be offered</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>UKI's own expert: movement in garden is landslip from removal of retaining land — not subsidence to main building; recommended low-level retaining wall. Consumer: cannot obtain subsidence cover elsewhere; UKI's expert identified the exact problem. FOS investigator: ABI continuation guidance applied; UKI should stand by its own expert's findings. FOS ombudsman: ABI guidance not strictly relevant (claim declined; no repairs undertaken); key issue is whether UKI correctly applied its underwriting criteria — underwriting guide specifies 'subsidence' not 'landslip'; UKI's own expert found landslip not subsidence; policy separately defines subsidence, ground heave and landslip as distinct events; UKI has not demonstrated it applied its criteria correctly to the identified peril</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>UKI to reinstate and backdate subsidence cover for the 2023–2024 policy period, subject to Mrs and Mr A paying any relevant additional premium; pay £150 compensation for unnecessary inconvenience</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P24" s="3" t="inlineStr">
+        <is>
+          <t>Insurer's underwriting criteria must be correctly applied to each identified peril — where criteria specifically address 'subsidence' and not the broader SHL perils (subsidence, heave, landslip), insurer cannot rely on those criteria to remove subsidence cover when its own expert identified the peril as landslip; subsidence and landslip are distinct perils (both in fact and under policy terms that list them separately) and must be treated accordingly in underwriting decisions; insurer whose own investigation identified the cause as landslip is bound by that finding and cannot invoke subsidence criteria to remove subsidence cover; the plain text of an underwriting guide is the primary indicator of what action was authorised — insurer's assertion of a broader interpretation is insufficient</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>Whether UKI's underwriting guide's reference to 'subsidence' was intended to encompass all three SHL perils or only subsidence specifically (UKI asserted broader scope; FOS found plain text did not support this)</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>UKI's own expert confirmed landslip not subsidence; UKI's underwriting guide says subsidence cover declined for signs of or suffering subsidence — not for landslip; policy terms list three distinct events (subsidence, ground heave, landslip) confirming they are separate; UKI's argument that 'subsidence' in the guide meant all three perils is not supported by plain text; UKI has not demonstrated it applied its criteria correctly; subsidence cover must be reinstated; £150 for inconvenience of being unable to obtain subsidence cover elsewhere</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>When an insurer's own expert investigation identifies the damage as landslip rather than subsidence, that finding binds the insurer's subsequent underwriting decisions about each named peril — the insurer cannot then invoke subsidence criteria to remove subsidence cover; underwriting guides that use the word 'subsidence' do not automatically extend to landslip or heave unless the guide explicitly says so; each of the three SHL perils must be assessed independently in underwriting and claims decisions; the ABI continuation guidance may not apply when a claim has been declined and no repairs undertaken, but the insurer must still correctly apply its own criteria to each specific peril</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>IF insurers_expert_identifies_peril_as_landslip_not_subsidence THEN insurer_cannot_invoke_subsidence_underwriting_criteria_to_remove_subsidence_cover; subsidence_and_landslip_are_distinct_perils_that_must_be_assessed_independently_in_underwriting_and_claims; IF underwriting_guide_refers_to_subsidence_only THEN it_does_not_authorise_action_based_on_landslip_or_heave_unless_expressly_stated; insurer_is_bound_by_the_plain_text_of_its_underwriting_guide_broader_interpretation_requires_explicit_textual_support</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5220010.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="120" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-024</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5315100</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>9 Jul 2025</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance — subsidence claim accepted February 2021 (tree root clay soil shrinkage; vegetation removed); multi-year dispute about ongoing movement monitoring, drain repair coverage, AXA removing subsidence cover at renewal (admitted breach of ABI guidance), cash settlement management fee deduction, and delay and poor communication over approximately three years; claim still not at repair stage at date of decision</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Tree root-influenced clay soil shrinkage (vegetation removed 2021 and further tree identified January 2025 and removed); drain damage also identified but AXA disputes connection to subsidence; movement ongoing during multi-year claim period</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>AXA: property stabilised post-vegetation removal; damaged drains not caused by or contributing to subsidence (cyclical not progressive movement — not drain-related subsidence); management fee deduction from cash settlement in line with policy terms (payment capped at what AXA would pay preferred supplier, excluding management coordination costs); subsidence cover removal situation under investigation</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Mrs R: consumer-commissioned monitoring shows continued movement; surveyor says drains could be a cause; chip board flooring damaged by subsidence. AXA: cyclical not progressive movement — not drain-related; purchase survey showed flooring distortion predating subsidence; management fee is a non-repair cost excluded from cash settlement. FOS (provisional): further monitoring needed; drain reimbursement requires specific expert evidence not yet available; £1,500 excess management fee deduction is fair per policy terms; £1,500 compensation for multi-year delay. FOS (final): AXA accepted breach of ABI continuation guidance; Jan 2025 neighbour's tree removed; ongoing monitoring continuing; floor damage not conclusively subsidence-related; drain expert evidence not provided — AXA's position (cyclical movement) accepted in absence of contradicting evidence; three years continuing cover from final COSA date directed</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>AXA to arrange subsidence cover on reasonable terms (as part of full buildings insurance policy) for a minimum of three years from the date of issue of a final Certificate of Structural Adequacy (COSA); pay Mrs R £1,500 compensation for distress and inconvenience from multi-year delay</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>ABI continuation guidance on subsidence cover extends beyond claim conclusion and the repair period — the obligation to provide continuing cover applies after a final COSA is issued (post-repair), not merely until the claim is administratively closed; minimum three years cover from final COSA provides assurance to the housing market and to the consumer without creating an unlimited obligation; insurer removing cover at claim conclusion acts inconsistently with the guidance's purpose; cash settlement for subsidence repairs is capped at what insurer would pay its own preferred supplier — management/coordination costs are non-repair costs and are legitimately excluded; expert evidence specific to the dispute is required before FOS will direct reimbursement of drain costs — consumer's surveyor suggestion is insufficient; insurer dispute about repair method (underpinning vs resin injection) is not within FOS competence to direct — insurer's chosen method is acceptable if effective</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>Expert evidence specifically linking drain damage to the subsidence movement (not provided — FOS could not direct drain cost reimbursement); confirmation of whether chip board flooring distortion predated subsidence or was caused by it (purchase survey noted pre-existing distortion); AXA's underwriter explanation for subsidence cover removal (never provided — AXA ultimately accepted breach)</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>AXA accepted approximately seven months of attributable delay in the period reviewed; £1,500 compensation appropriate given Mrs R's health circumstances and her son's health, and the extended claim life; ABI continuation guidance 'after the repair is effected' language means cover continues post-repair, not that cover ceases at claim closure; three years from final COSA is proportionate and not unreasonably open-ended; management fee: policy says payment will not exceed amount AXA would pay preferred supplier — management fee is excluded as a non-repair cost, and £1,500 deduction is fair; floor distortion: purchase survey noted pre-existing unevenness — insufficient evidence subsidence worsened beyond that; drains: AXA's position (cyclical not progressive movement) accepted in absence of contradicting expert evidence from consumer</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>ABI continuation guidance must be read as extending beyond claim closure to the post-repair period — insurer removing subsidence cover when a claim concludes acts against the guidance's purpose; minimum cover period of three years from issue of final COSA is a proportionate industry-consistent obligation; cash settlement for subsidence repairs may legitimately exclude insurer management and coordination fees as non-repair costs within the policy's cash settlement cap; consumer must produce specific expert evidence linking a disputed damage element (drains, flooring) to subsidence before FOS will direct reimbursement — a surveyor's unsubstantiated suggestion is not sufficient</t>
+        </is>
+      </c>
+      <c r="T25" s="5" t="inlineStr">
+        <is>
+          <t>ABI_continuation_guidance_extends_beyond_claim_closure_to_post_repair_period; minimum_three_years_cover_from_final_COSA_is_proportionate_continuing_cover_obligation; cash_settlement_for_subsidence_repairs_may_exclude_insurer_management_fees_as_non_repair_costs; IF consumer_claims_drain_or_other_element_is_subsidence_related THEN specific_expert_evidence_required_before_FOS_will_direct_reimbursement; IF insurer_removes_subsidence_cover_at_claim_conclusion THEN removal_is_inconsistent_with_ABI_continuation_guidance</t>
+        </is>
+      </c>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5315100.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="120" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5375880</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Highway Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>23 Apr 2025</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Buildings insurance — new cracking August 2022; Highway avoided policy citing careless misrepresentation on 'Is the property and surrounding area free from subsidence?' answered 'Yes'; property had a prior 2003 subsidence claim (tree roots; same beech tree implicated in both incidents) but repairs carried out then and no further signs for nearly 20 years; beech tree is local authority property and cannot be removed</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Tree root-induced subsidence (same local authority beech tree identified as cause of both 2003 and 2022 incidents); 2003 repairs included root barrier, drain replacement, and wall stitching; no further movement observed for nearly 20 years between the two incidents</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Highway: property not 'free from subsidence' because the tree identified as the cause of both incidents was present and unremoved at inception; 2003 stitch repairs stabilised cracking but did not remove the cause of the subsidence; consumer should have answered 'No' to the question; careless misrepresentation at inception entitles avoidance under CIDRA 2012</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Mr and Mrs D: 2003 repairs were substantial (root barrier, drain replacement, wall stitching); no further subsidence signs for nearly 20 years; reasonably believed subsidence had been resolved; question did not ask about previous subsidence claims; tree is local authority property — cannot be removed. Highway: stitch repairs only stabilised not resolved the cause; tree still present means property is not free from subsidence; should have answered 'No.' FOS: question does not define 'property' or 'surrounding area'; no timeframe or geographic scope given; no guidance on how to answer if property was previously affected; question did not ask about prior subsidence claims specifically; consumer who carried out substantial repairs in 2003 and experienced no further movement for nearly 20 years reasonably believed the subsidence was resolved; presence of an unremovable local authority tree does not automatically mean the property is currently 'affected by subsidence'; CIDRA reasonable care test met</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>Highway to reinstate policy and deal with the subsidence claim in line with remaining policy terms and conditions; consumer may need to repay any premiums that were previously refunded following avoidance</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>CIDRA 2012 — consumer must take reasonable care not to misrepresent; where a question about subsidence does not define the geographic scope of 'property and surrounding area', provide a timeframe, or give guidance for consumers who previously experienced subsidence, the insurer cannot establish that reasonable care was not taken; consumer who carried out substantial post-subsidence repairs and experienced no further movement for nearly 20 years reasonably believes the subsidence is resolved; presence of an unremovable third-party tree does not automatically mean the property is currently affected by subsidence; insurer cannot extend the meaning of its vague question beyond what a reasonable consumer would understand it to mean; statement of fact that does not include a prior claims question cannot be relied upon to show the consumer should have disclosed prior subsidence history</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>Whether the statement of fact specifically asked about prior subsidence claims (FOS found it did not); precise intended scope of 'property and surrounding area free from subsidence' (insurer failed to define this at time of application)</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
+          <t>2003 repairs were substantial — root barrier, drains replaced, walls stitched; no further damage for nearly 20 years; consumers reasonably believed subsidence was resolved; statement of fact did not ask about prior subsidence claims; question 'free from subsidence' has no defined scope, timeframe or guidance for previously affected properties; Highway did not prove the question was asked in a way that meant the consumer should have answered 'No'; presence of unremovable local authority tree does not automatically mean property is currently affected; CIDRA reasonable care test met; avoidance is not available to Highway</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>Insurer relying on CIDRA to avoid a policy for non-disclosure of prior subsidence must show that the question asked was clear enough that a reasonable consumer would know the correct answer — a question with no geographic scope, no timeframe and no guidance for previously affected properties is too vague to support an avoidance; consumer who completed substantial post-subsidence repairs and experienced no further movement for nearly 20 years has reasonable grounds to believe the subsidence was resolved; insurer cannot treat the continued presence of an unremovable third-party tree as conclusive evidence that the property is 'affected by subsidence' for disclosure purposes</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>CIDRA_reasonable_care_test_requires_question_to_be_clear_enough_that_consumer_would_know_correct_answer; IF question_about_subsidence_has_no_defined_scope_or_timeframe THEN insurer_cannot_establish_consumer_failed_reasonable_care_standard; IF substantial_post_subsidence_repairs_carried_out AND no_further_movement_for_twenty_years THEN consumer_reasonably_believes_subsidence_is_resolved; presence_of_unremovable_third_party_tree_does_not_automatically_mean_property_is_currently_affected_by_subsidence; statement_of_fact_without_prior_claims_question_cannot_support_non_disclosure_of_prior_subsidence_history</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5375880.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="120" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-026</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5643066</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Ageas Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>12 Nov 2025</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Landlord insurance — subsidence discovered August 2022 (policy inception October 2021); Ageas initially accepted claim; reversed and declined in August 2024 on grounds damage predated inception; relied on September 2021 tenancy check-in report (uPVC doors could not fully close) and 2015 survey noting signs of settlement; window specialist confirmed door issue was unrelated to subsidence; ongoing movement confirmed at August 2023 revisit</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Subsidence caused by effect of nearby vegetation on clay soil (identified by loss adjuster October 2022 — moderate to severe cracking internally and externally); new damage areas observed at August 2023 revisit confirming ongoing movement during policy period</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Residential let property (landlord insurance; limited company policyholder — FOS for small businesses jurisdiction)</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Pre-Inception Damage Dispute</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Ageas (first response): cracking appeared prior to inception; 2015 survey showed signs of settlement/subsidence not disclosed on Statement of Facts. Ageas (second response): September 2021 check-in report showed two uPVC doors could not close fully — evidence of pre-inception subsidence; claim predated start of cover</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Loss adjuster (October 2022): moderate to severe cracking; damage arose during currency of policy; new damage areas at August 2023 revisit. Check-in report (September 2021): 43 pages — no mention of structural cracking; two uPVC doors noted as not closing fully. Window/conservatory repair specialist: uPVC doors unaffected by subsidence; frames straight and flush; door catching is weather-related and needs servicing/adjustment. Decorator's quote (September 2021): mentioned filling cracks before letting but no structural concerns raised. FOS: check-in report does not mention cracks that were later observed; uPVC door issue confirmed unrelated to subsidence by specialist; decorator did not raise structural concerns; loss adjuster confirmed insurable interest and damage during policy currency; some pre-policy cracks possible but Ageas cannot differentiate between pre- and post-inception subsidence damage</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>Ageas to deal with subsidence claim in line with policy terms; assess claim for loss of rental income; reinstate policy if cancelled; pay P £800 compensation for impact on rental income and inability to let the property</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="n">
+        <v>800</v>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P27" s="5" t="inlineStr">
+        <is>
+          <t>For a subsidence claim decline to succeed entirely on pre-existing damage grounds, insurer must show that the subsidence damage both started and stopped before policy inception — if subsidence began before inception but continued during the policy period, insurer must deal with the claim; where insurer cannot differentiate between pre-inception subsidence damage and post-inception damage, FOS requires insurer to deal with all the subsidence damage; an insurer that accepts a claim at first assessment and later reverses that acceptance on the same facts must show clearly that the reversal is justified; insurer that affirms a contract by issuing a second final response focused solely on a new ground (uPVC doors) may be treated as having abandoned the earlier ground (IA 2015 fair presentation breach) and cannot later revive it</t>
+        </is>
+      </c>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>Pre-policy structural survey specifically recording cracking extent (none available — no pre-policy structural survey of crack damage existed); whether the 2015 survey settlement/subsidence findings represented active ongoing subsidence or a resolved historic issue</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>Check-in report (43 pages) does not mention any of the cracks later identified; uPVC door issue confirmed unrelated to subsidence by specialist — frames straight and flush; decorator quote mentioned filling cracks without raising structural concerns; loss adjuster confirmed claim arose during policy currency and moderate-to-severe cracking was found; new damage areas at 2023 revisit confirm ongoing movement during policy; some pre-policy cracks may exist but Ageas cannot differentiate — must deal with all subsidence damage; Ageas appeared to have accepted the fair presentation explanation by issuing second final response focused only on uPVC doors; £800 for impact on rental income and inability to let the property</t>
+        </is>
+      </c>
+      <c r="S27" s="5" t="inlineStr">
+        <is>
+          <t>Insurer relying on pre-inception damage to decline a subsidence claim must show not only that some damage may have existed before inception but also that the current damage is entirely attributable to pre-inception movement — if subsidence was ongoing at inception and continued during the policy, the insurer must deal with the claim; where specific evidence (check-in report, decorator's quote) does not in fact show structural cracking, it cannot support a pre-inception damage exclusion argument; a specialist confirmation that an alleged sign of subsidence (uPVC door catching) is in fact weather-related is binding on the insurer unless contradicted by other expert evidence; insurer that issues a second final response focused on a new ground may be taken to have affirmed the contract on the original ground</t>
+        </is>
+      </c>
+      <c r="T27" s="5" t="inlineStr">
+        <is>
+          <t>IF subsidence_began_before_inception_but_continued_during_policy THEN insurer_must_deal_with_claim; IF insurer_cannot_differentiate_pre_and_post_inception_subsidence_damage THEN insurer_must_deal_with_all_damage; alleged_sign_of_subsidence_confirmed_by_specialist_as_unrelated_to_subsidence_cannot_support_pre_inception_exclusion; IF insurer_issues_second_final_response_focused_on_new_ground THEN may_be_taken_as_affirmation_abandoning_first_ground; pre_inception_damage_exclusion_requires_evidence_damage_started_and_stopped_before_inception</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5643066.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="120" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5656370</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>30 Jul 2025</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Property protection insurance (block of flats) — subsidence claim accepted 2020; AXA increased premium by 110% at 2023 renewal and removed subsidence cover when its commercial arrangement with intermediary T ended and it applied different underwriting criteria; policyholder C unable to access open market due to ongoing claim; excess increase from £1,500 to £5,000 also proposed without supporting evidence</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Subsidence (cause not specified — accepted 2020; claim ongoing and not resolved at time of decision)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Block of flats (property protection insurance; commercial policy — FOS for small businesses jurisdiction; FOS applied good industry practice principles equivalent to domestic guidance)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>AXA: 2021 and 2022 premium increases reflected general pricing factors; 2023 premium reflects new underwriting criteria applied when direct policy offered following end of arrangement with T; subsidence cover cannot be offered as claim is ongoing and property stability unconfirmed; at 2023 renewal AXA was applying different (higher risk) criteria than those used under the T arrangement</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>C: some increase expected but 110% while also removing subsidence cover is excessive and unfair; trapped with AXA due to ongoing claim and unable to move to another insurer. AXA (initial): limited evidence for increases. AXA (later): 2021/22 increases due to inflation, index linking, general risk changes — not claim-driven; subsidence cover removal due to claim being ongoing. FOS: 2021/22 increases fair (market-consistent, not claim-driven, subsidence cover maintained); 2023 increase unfair — AXA switched from T-arrangement criteria to its own higher-risk criteria without considering C's inability to access the open market; AXA cannot use its own unresolved claim to justify removing cover it is handling; excess increase to £5,000 proposed without underwriting rationale or evidence — rejected</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>AXA to reduce 2023 premium to £6,500 (approximately 20% increase consistent with 2021–22 approach) and refund difference plus 8% simple interest; reduce 2024 premium to £6,825 and refund difference plus 8% simple interest; reinstate subsidence cover for 2023 and 2024 without additional premium or excess increase beyond £1,500; pay £200 compensation for prolonged inconvenience</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>Insurer that changes its underwriting criteria because of a change in commercial arrangements (e.g. end of intermediary agreement) must consider the impact on policyholders who cannot access the open market due to an ongoing claim; a policyholder with an open subsidence claim is effectively locked in to the incumbent insurer and cannot obtain alternative cover on normal terms — the insurer cannot exploit that lock-in by applying materially different criteria; insurer handling a subsidence claim cannot remove subsidence cover on grounds that it has not resolved its own claim — the insurer's own handling failure cannot be used to disadvantage the policyholder; excess increases proposed without supporting underwriting evidence or rationale will not be accepted by FOS</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>AXA's calculation of what 2023 and 2024 premiums would be under the 2021–22 approach (AXA never provided this despite multiple opportunities — FOS derived the 20% figure from the two prior year average)</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>2021 and 2022 increases market-consistent (inflation, index-linking, general risk changes) — not claim-driven; subsidence cover maintained; these increases were fair. 2023 increase of 110% — consequence of end of T arrangement and application of different higher-risk criteria; AXA should have considered C's inability to access open market; increase is unfair. Subsidence cover removal — AXA, as claim handler, cannot say its own unresolved claim makes the risk too great to cover; AXA itself offered reinstatement in earlier discussions. Excess increase to £5,000 proposed with no supporting evidence or underwriting rationale — rejected. £200 compensation for prolonged inconvenience</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="inlineStr">
+        <is>
+          <t>When an insurer's underwriting criteria change because of a change in commercial or distribution arrangements, it must consider the impact on policyholders who are locked in because of ongoing claims — applying substantially harsher criteria to a policyholder who has no realistic alternative is unfair; insurer handling a claim cannot use its own delay or non-resolution of the claim as justification for removing cover that it was providing — a claim that remains open is not a reason to remove the very cover that applies to the claim; excess or premium increases proposed without underwriting evidence will be disregarded by FOS regardless of whether the increase itself may be technically justified</t>
+        </is>
+      </c>
+      <c r="T28" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_changes_criteria_due_to_change_in_commercial_arrangements AND policyholder_cannot_access_open_market_due_to_ongoing_claim THEN applying_materially_harsher_criteria_is_unfair; IF insurer_handling_subsidence_claim_removes_subsidence_cover_citing_unresolved_claim THEN removal_is_unfair_as_insurer_cannot_use_own_handling_failure_to_disadvantage_policyholder; excess_increases_without_supporting_underwriting_evidence_or_rationale_will_be_rejected_by_FOS; premium_increases_must_be_consistent_with_market_approach_not_driven_by_change_in_commercial_distribution_arrangement</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5656370.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="120" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-028</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5718419</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>West Bay Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>25 Dec 2025</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Property owners insurance (block of leasehold flats) — subsidence claim accepted 2018; West Bay withdrew its property owners policy product at 2019 renewal and subsequently withdrew from the buildings insurance market entirely; T (limited company managing the building) left without subsidence cover from 2019 to 2025 (approximately six years) until a Certificate of Structural Adequacy was issued; West Bay took no steps to arrange alternative cover or mitigate impact</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Subsidence (cause not specified — accepted claim 2018; repairs completed early 2023; final COSA issued 2025)</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Block of leasehold flats (property owners policy; limited company managing building — FOS considered distress of individual leaseholders within the company)</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>West Bay: withdrew property owners policy product at 2019 renewal as a commercial decision; subsequently withdrew from buildings insurance market entirely; obligation to offer continuing cover applies but was not possible due to market withdrawal; extension of cover would require maintaining a product withdrawn from all policyholders of that type</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>T: West Bay should have taken steps to ensure continuing subsidence cover was available; without accepted claim insurer's assistance, finding alternative cover with subsidence inclusion is extremely difficult or impossible; six years without subsidence cover caused significant concern and administrative burden. West Bay: market withdrawal is a commercial necessity applicable to all such policyholders; T was informed and had time to seek alternative cover; £1,000 compensation offered. FOS: West Bay acknowledged the general continuing cover obligation; should have explored options (similar product, maintaining cover until claim complete, arranging block transfer to another insurer); West Bay took no steps beyond not renewing; no new subsidence claims arose during gap period; financial loss from premiums unlikely (subsidence claim would have meant substantially higher premiums for any cover obtained); £1,000 compensation appropriate for six years of concern and administrative burden</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>West Bay Insurance Plc to pay £1,000 compensation for six years of distress and inconvenience caused by being left without subsidence cover</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P29" s="5" t="inlineStr">
+        <is>
+          <t>When an insurer withdraws its product or exits the market, it must consider the likely detriment to policyholders with ongoing or recently settled subsidence claims and take steps to mitigate it — acceptable steps include offering a similar product, maintaining cover until the claim is complete, or arranging for another insurer to step in; this obligation applies regardless of whether the withdrawal applies to all policyholders of that product type or just one; failure to explore any of these options before withdrawing leaves policyholders without cover, contrary to good industry practice; where no new subsidence claims arise during the period without cover, financial loss is unlikely; compensation for distress and administrative inconvenience is the primary remedy</t>
+        </is>
+      </c>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>What steps West Bay could have taken to arrange alternative cover or a block transfer for T (never explored by West Bay); whether a block transfer to another insurer was feasible given the market at that time</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="inlineStr">
+        <is>
+          <t>West Bay was aware of the continuing cover obligation; took no steps to mitigate the impact on T; T unable to find subsidence cover elsewhere for six years; no new subsidence claims arose during the gap — financial loss is unlikely; higher premiums would have been likely if subsidence cover had been obtained; £1,000 fair and in line with FOS approach for six years of concern and administrative burden</t>
+        </is>
+      </c>
+      <c r="S29" s="5" t="inlineStr">
+        <is>
+          <t>When an insurer withdraws a product that covers policyholders with active or recently settled subsidence claims, it must proactively explore options to protect those policyholders before the cover lapses — simply not renewing the policy is insufficient; acceptable measures include maintaining the specific policy until the claim concludes, arranging a block transfer to another insurer, or offering a comparable product; insurer must actively investigate whether alternatives are possible before concluding that market withdrawal makes continuing cover impossible; where no financial loss results from the period without cover, compensation for distress and inconvenience remains the appropriate and primary remedy</t>
+        </is>
+      </c>
+      <c r="T29" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_withdraws_product_or_exits_market AND policyholder_has_open_or_recent_subsidence_claim THEN insurer_must_explore_steps_to_mitigate_detriment_before_cover_lapses; acceptable_mitigation_steps_include_maintaining_policy_until_claim_complete_OR_arranging_block_transfer_OR_offering_comparable_product; simply_not_renewing_the_policy_is_not_adequate_mitigation; IF_no_new_claims_arise_during_gap_period THEN_financial_loss_is_unlikely_but_distress_and_inconvenience_compensation_remains_appropriate; obligation_applies_regardless_of_whether_withdrawal_affects_all_policyholders_of_that_product_type</t>
+        </is>
+      </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5718419.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="120" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5755602</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Saga Services Limited</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>12 Sep 2025</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Buildings insurance — Saga (broker) moved Mrs C's policy from insurer A to insurer B at renewal without pausing to consider a subsidence issue Mrs C had reported three days before renewal; insurer A subsequently had no continuing cover obligation; insurer B removed subsidence cover when it discovered the claim at renewal three; Mrs C left without subsidence cover despite an ongoing subsidence claim with insurer A</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Subsidence (cause not specified — ongoing claim with insurer A; new episodes would not be covered under current policy with C)</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Saga: first record of Mrs C's subsidence issue was after renewal two (contradicted by call transcript); no internal process to contact insurer A or prevent policy moving; cannot force panel insurers to provide cover; at renewal three adequately disclosed the subsidence cover exclusion</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Mrs C: told Saga about cracks three days before renewal two (call 12 December); Saga should have paused the renewal and contacted insurer A. Saga: no record of subsidence call before renewal two; no process for involving A. FOS: call transcript confirms Mrs C clearly reported cracks on 12 December before renewal two and was referred to insurer A; Saga had a working relationship with A at renewal two and should have paused the renewal to notify A; insurer A would more likely than not have renewed given industry continuing cover guidance; Saga's inaction broke the chain of cover; at renewal three Consumer Duty required much clearer communication than a generic reference to excluded perils — Saga's own later letter acknowledged its communication at renewal three was inadequate; £2,000 compensation</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>Saga Services Limited to pay Mrs C £2,000 compensation for distress and inconvenience from loss of subsidence cover and ongoing difficulty obtaining replacement cover</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>Broker who is notified by a consumer of a subsidence issue (crack report) before a renewal must take action to protect the consumer's continuing subsidence cover — the broker must not allow the policy to move to a new insurer without flagging the issue to the current insurer; broker's internal process limitations or panel structure are not an excuse for inaction that causes consumer harm; Consumer Duty (and ICOBS 8 equivalent) requires brokers to ensure consumers understand significant coverage limitations — a generic reference to 'exclusions may apply' is insufficient to notify a consumer that subsidence cover has been removed; once a broker's inaction breaks the chain of continuing cover, the consumer loses the protection that industry guidance was intended to preserve</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>Whether insurer A would specifically have renewed Mrs C's policy had Saga contacted them (FOS found it more likely than not A would have renewed given industry continuation guidance); full extent of financial loss from broken cover chain (could not be fully quantified given involvement of insurer A's future decisions)</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>Call transcript contradicts Saga's claim that no prior record existed — Mrs C clearly reported cracks on 12 December before renewal two and was referred to insurer A; Saga had a working relationship with A at that time and should have paused the renewal; A would more likely than not have renewed given industry continuing cover guidance; Saga's inaction broke the chain — A had no obligation at renewal three; B was a different insurer with no continuing cover obligation; Saga also failed at renewal three under Consumer Duty (generic exclusion reference plus no follow-up call was inadequate); Saga's own letter acknowledging inadequate communication at renewal three is an admission; £2,000 appropriate for distress and ongoing difficulty obtaining subsidence cover</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>Broker who learns of a subsidence issue from a consumer before renewal must pause the renewal process and contact the incumbent insurer — allowing the policy to roll to a new insurer automatically when a subsidence issue has been reported is a breach of the broker's duty to act in the consumer's best interests; the broker's internal workflow or panel limitations do not override this duty; when subsidence cover is excluded from a new policy as a consequence of the broker's action or inaction, the consumer must be given specific and prominent notification of that exclusion in plain terms, not a generic reference to possible exclusions</t>
+        </is>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>IF broker_notified_of_subsidence_issue_before_renewal THEN broker_must_pause_renewal_and_contact_incumbent_insurer; broker_internal_process_limitations_do_not_excuse_inaction_causing_consumer_harm; IF broker_inaction_breaks_chain_of_continuing_subsidence_cover THEN broker_is_liable_for_D_and_I_and_consequential_cover_loss; consumer_duty_requires_specific_prominent_notification_of_subsidence_cover_exclusion_not_generic_reference_to_excluded_perils</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5755602.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="120" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-030</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>DRN-6019596</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>11 Jan 2026</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Landlord HMO buildings insurance (AXA PrimeLet) — subsidence claim January 2023; AXA wrongly told Ms L in July 2024 that damage to the front of her property was not subsidence-related; by August 2024 AXA knew the front was a separate subsidence incident from the rear (different cause) but never set up a new claim; avoidable delay of several months and poor communication throughout; consumer commissioned independent structural engineer (£600) after receiving inconsistent explanations</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Two separate subsidence incidents: rear of property — defective drainage causing ground movement (investigation concluded June 2024; rear claim resolved); front of property — clay shrinkage from vegetation (separate cause; separate claim required; not resolved at time of decision)</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>HMO (House in Multiple Occupation) let property (AXA PrimeLet commercial landlord policy)</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>AXA: front of property damage not subsidence-related (July 2024 position — later reversed in August 2024); two separate subsidence events with different causes require two separate claims and two policy excesses; communication acknowledged as poor</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>Ms L: subsidence across the whole structure; AXA's surveyor gave inconsistent explanations without having visited the property; AXA should automatically set up a new claim for the front. AXA's surveyor (July 2024): front crack pattern does not indicate subsidence — outside scope. Ms L's independent structural engineer (£600): front = subsidence from clay shrinkage from nearby vegetation; rear = subsidence from damaged underground pipe; bathroom damage likely not subsidence-related. AXA (August 2024): reversed July 2024 position — front is a separate subsidence incident. FOS: AXA was wrong to tell Ms L in July 2024 that the front was not subsidence-related; once AXA knew in August 2024, it should have set up a new claim immediately — this was never done; avoidable delay of several months from July to October 2024 when rear repairs could have started but did not; two different causes = two separate claims and two excesses is fair; £1,500 total D&amp;I compensation; £600 engineer cost refundable</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>AXA to increase total compensation to £1,500 (additional £1,150 on top of £350 already offered); reimburse Ms L for independent structural engineer's report cost of £600 plus 8% simple interest from date of payment to date of settlement</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P31" s="5" t="inlineStr">
+        <is>
+          <t>When an insurer's own investigation reversal confirms that a previously excluded area is in fact subsidence, the insurer must proactively set up a new claim immediately — it cannot wait for the consumer to initiate the new claim; where a consumer receives inconsistent information from an insurer (exclusion reversed within weeks), the consumer who commissions independent professional evidence to resolve the inconsistency is entitled to reimbursement of that cost; two subsidence incidents with different identified causes are properly treated as two separate claims with two policy excesses; avoidable delay in progressing an accepted subsidence claim (where repairs could have begun but did not due to insurer's handling failures) is compensable</t>
+        </is>
+      </c>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>Whether AXA's surveyor had visited the front of the property before giving the July 2024 advice that the front was not subsidence-related (AXA's surveyor appeared not to have done so); precise timeline of when AXA's August 2024 reversal was communicated to Ms L</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>AXA was wrong to tell Ms L in July 2024 that the front was not subsidence-related — AXA itself reversed this within weeks in August 2024; once AXA knew the front was a separate subsidence incident it should have set up a new claim immediately; this was never done; avoidable delay of several months for the rear repairs (could have started July 2024 but did not until October 2024); Ms L was left with inconsistent explanations and had no realistic choice but to commission an independent engineer; engineer cost of £600 reimbursable; two different causes = two separate claims and two excesses is fair and not contested further by FOS; £1,500 total D&amp;I compensation appropriate given duration of delay and inconvenience</t>
+        </is>
+      </c>
+      <c r="S31" s="5" t="inlineStr">
+        <is>
+          <t>When an insurer's investigation reverses a prior exclusion decision (e.g. front of property initially excluded as not subsidence, then confirmed as subsidence), the insurer must immediately set up the new claim without waiting for the consumer to re-initiate it — failure to do so creates both an avoidable delay and a liability for consequential costs; where a consumer receives conflicting technical advice from the insurer over a short period and commissions independent engineering evidence to resolve the inconsistency, the insurer must reimburse that cost; two simultaneously identified subsidence incidents with different identified causes are properly treated as two separate claims with separate excesses — this position is defensible provided it is explained clearly and promptly</t>
+        </is>
+      </c>
+      <c r="T31" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_reverses_exclusion_and_confirms_area_is_subsidence THEN insurer_must_proactively_set_up_new_claim_without_waiting_for_consumer; IF consumer_commissions_independent_engineer_to_resolve_inconsistent_insurer_advice THEN insurer_must_reimburse_engineer_cost; two_subsidence_incidents_with_different_identified_causes_may_be_treated_as_two_separate_claims_with_two_excesses; avoidable_delay_in_progressing_accepted_subsidence_claim_due_to_insurer_handling_failure_is_compensable</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>DRN-6019596.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add SUBS-031 to SUBS-032 to Subsidence Case Database — Batch 4 complete (Subsidence database final)
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Subsidence_Case_Database.xlsx
+++ b/knowledge/case-databases/Subsidence_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3753,6 +3753,216 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="120" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>SUBS-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>DRN8130715</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>15 Jul 2015</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — 2009 subsidence claim recorded against extension crack (clay shrinkage from willow tree); repair cost below £1,000 policy excess so no contractor repairs carried out; UKI failed to explain to Mr A that not proceeding with insurer-managed repairs meant no Certificate of Structural Adequacy would be issued; Mr A unable to sell home or insure elsewhere; dispute about removal of subsidence record and insurer's obligation to provide COSA</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Clay shrinkage from willow tree (high water demand) causing minor subsidence to extension/main house junction in 2009; willow tree pruned and chemically treated as mitigation; property stabilised by 2013 with no recent or progressive subsidence found at 2013 inspection</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>UKI: 2009 subsidence correctly recorded (loss adjuster's local knowledge; willow tree; tapering crack; ten years since extension built so not settlement); repair cost fell below £1,000 excess so not carried out; willow tree pruned and chemically treated as mitigation; property since stabilised; 2013 engineer report confirms no current subsidence; Certificate of Structural Adequacy only issued after contractors complete physical repairs — no repairs = no COSA; modified engineer's report provided instead</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Mr A: loss adjuster's 2009 investigation was superficial (no inspection trench, no monitoring); 2013 engineer report found no evidence of recent, historic or ongoing subsidence — proves 2009 recording was wrong; two cracks still same size and shape proving they were never subsidence; UKI told him damage was repaired but no repairs were carried out. UKI: loss adjuster's local knowledge and willow tree justified classification; damage recovered and no further movement proves cause correctly identified; 2013 report confirms no current subsidence; not required to remove valid claim. FOS adjudicator: 2009 investigation should have been more detailed; but subsidence recording reasonable given local knowledge, tapering crack, willow tree. FOS ombudsman: on balance minor subsidence did occur in 2009 — local knowledge, slight tapering, 10 years since extension (settlement less likely), willow tree nearby; UKI investigation poor — no monitoring, no in-depth investigation; cannot direct removal of valid subsidence claim; 2013 report finding no current subsidence does not prove the 2009 cracks were not subsidence; UKI's provided engineer's report was inadequate (cut-and-paste from 2013 report with 'historic' inserted); COSA is appropriate remedy</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited to provide Mr A with a Certificate of Structural Adequacy in respect of the 2009 claim; pay £500 compensation for distress and inconvenience caused by poor handling of subsidence claim</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr">
+        <is>
+          <t>Where a subsidence claim is accepted but repair cost falls below the policy excess and no contractor repairs are carried out, the insurer must explain to the consumer that not proceeding with insurer-managed repairs means no Certificate of Structural Adequacy will be issued; failure to give this warning causes lasting harm (inability to sell, inability to move insurer) for which the insurer is responsible; the appropriate remedy is to provide a genuine COSA or to fund an independent structural engineer's report acceptable to future insurers and purchasers; FOS cannot direct removal of a valid subsidence claim from records even if the original investigation was poor — the remedy is to address the consequences of poor handling, not to re-characterise the claim history; chemically treating and pruning vegetation (even if not physically removed) constitutes remedial work; an inadequate document cut-and-pasted from a prior report does not satisfy the insurer's obligation to provide a COSA-equivalent document</t>
+        </is>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>Physical inspection trench or monitoring data from the 2009 claim (loss adjuster did not carry out any in-depth investigation); full engineer's January 2015 report (only conclusion page provided — confirmed to be restatement of 2013 inspection position rather than a new inspection)</t>
+        </is>
+      </c>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>On balance minor subsidence did occur in 2009 — loss adjuster's local knowledge of the area, slight tapering to the crack, ten years since the extension was built (making settlement a less likely cause) and the willow tree nearby; UKI's 2009 investigation was poor (no monitoring, no in-depth investigation, walked away from repairs because cost fell below excess); UKI failed to explain to Mr A that self-arranging the cosmetic repair and not paying the excess meant no COSA would be issued; this left him unable to sell or move insurer; 2013 engineer report finding no current subsidence does not prove the 2009 cracks were not subsidence — the property stabilised after tree treatment; UKI's offered 'structural engineer's report' was a cut-and-paste of the 2013 report with the word 'historic' inserted — inadequate and unhelpful; COSA is the correct remedy; £500 compensation appropriate for the lasting harm caused by poor handling</t>
+        </is>
+      </c>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>When a subsidence claim is accepted but repair costs fall below the policy excess, the insurer must actively explain to the consumer that self-managing cosmetic repairs without insurer-appointed contractors means no Certificate of Structural Adequacy will be issued — and must explain the lasting consequences of that (inability to sell; inability to move insurer); failure to give this warning at the time creates a liability that persists until the insurer provides a COSA or funds an independent report; FOS will not direct removal of a valid subsidence claim from records merely because the original investigation was poor — it will instead require the insurer to remedy the consequences; a substitute document that merely copies a prior inspection report does not satisfy the COSA obligation</t>
+        </is>
+      </c>
+      <c r="T32" s="3" t="inlineStr">
+        <is>
+          <t>IF subsidence_claim_accepted AND repair_cost_below_excess AND no_contractor_repairs THEN insurer_must_explain_that_no_COSA_will_be_issued_without_insurer_managed_repairs; IF insurer_fails_to_warn_of_COSA_consequence THEN insurer_must_provide_COSA_or_fund_independent_structural_engineers_report; FOS_cannot_direct_removal_of_valid_subsidence_claim_even_if_investigation_was_inadequate; inadequate_cut_and_paste_document_does_not_satisfy_COSA_obligation; chemical_treatment_and_pruning_of_vegetation_constitutes_remedial_work_even_if_vegetation_not_physically_removed</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>DRN8130715.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="120" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SUBS-032</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>DRN8561608</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>19 May 2016</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Residential Property Owners insurance (block of leasehold flats) — cover lapsed in 2013 when bank switched the policy to another insurer; Aviva was still dealing with a pre-2013 subsidence claim; new policy arranged with Aviva in 2014 but subsidence cover excluded; Aviva argued ABI domestic subsidence continuation guidance did not apply to D's commercially labelled policy; FOS rejected this and directed reinstatement of subsidence cover</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Subsidence (cause not specified — pre-2013 claim accepted and being dealt with by Aviva; claim not resolved when policy lapsed and new policy was issued without subsidence cover)</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Block of leasehold flats (Residential Property Owners insurance; D is a residents association/limited company; individual flat owners are directors/shareholders of D; building described by Aviva as 'occupied — residential property')</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>Aviva: not involved in the 2013 decision to switch to another insurer; ABI domestic subsidence continuation guidance applies only to domestic consumers — D's policy is commercial and the guidance does not apply; FOS exceeded its remit by applying domestic guidance to a commercial policyholder; entitled to decide what cover to offer; break in cover between 2013 and 2014 extinguishes any continuation obligation</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>D: Aviva was still dealing with a pre-2013 subsidence claim when cover was restructured; new policy should include subsidence cover as Aviva was the handling insurer. Aviva: ABI agreement only applies to domestic consumers; D's policy is commercial; not responsible for the 2013 lapse; entitled to decide what cover to offer. FOS provisional: the 2014 policy documents did not clearly exclude subsidence except in four specified circumstances; even if intended to exclude, the documents did not achieve this; good industry practice requires insurer dealing with subsidence claim to continue offering subsidence cover. FOS final: building is a residential block; Aviva's own schedules describe it as 'Residential Property Owners Insurance' and 'occupied — residential property'; individual flat owners are directors of D; ABI agreement applies to domestic properties owned and occupied in personal capacity — this effectively fits D; FOS also not restricted to ABI agreement — applies good industry practice regardless; Aviva provided no evidence D failed normal underwriting criteria; break in cover caused by third party does not affect the analysis; Aviva continued providing cover for 2014/15, 2015/16 and 2016/17 (even after provisional decision) — consistent with subsidence cover being appropriate</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited to continue providing cover for D's property including damage caused by subsidence, as long as D and/or its property meet its normal underwriting criteria other than for the risk of subsidence</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P33" s="5" t="inlineStr">
+        <is>
+          <t>ABI domestic subsidence continuation guidance applies where the building is effectively residential in nature — it is not disapplied merely because the policyholder is a residents association or limited company if the building is owned by individuals and used as private dwellings; where the insurer's own policy schedules describe the property as 'Residential Property Owners Insurance' and 'occupied — residential property', the policy effectively falls within the domestic guidance regardless of how the insurer categorises it commercially; FOS is not restricted to the terms of the ABI agreement — it applies good industry practice standards; where an insurer is dealing with a subsidence claim, good industry practice requires it to continue offering subsidence cover at renewal subject to normal underwriting criteria other than for subsidence risk; if the insurer asserts the policyholder or property fails its normal underwriting criteria, it must produce evidence of this; a break in cover caused by a third party's administrative decision does not extinguish the subsidence continuation obligation</t>
+        </is>
+      </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>Aviva's normal underwriting criteria evidence demonstrating that D or its property failed to meet those criteria (Aviva was asked to produce this and did not); clarification on whether Aviva settled the pre-2013 claim by undertaking to carry out or arrange repairs (Aviva did not provide this clarification despite being asked)</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="inlineStr">
+        <is>
+          <t>ABI agreement applies to domestic properties owned and occupied in personal capacity — building effectively fits this as it is a residential block owned by individual flat owners who are directors of D; Aviva's own schedules describe it as 'Residential Property Owners Insurance' and 'occupied — residential property'; ABI guidance applies; FOS also applies good industry practice beyond the strict ABI agreement; Aviva provided no evidence D failed normal underwriting criteria; break in cover in 2013 not caused by Aviva's actions and does not affect analysis; Aviva's continued provision of cover for 2014/15, 2015/16 and 2016/17 (even after objecting to provisional decision) is consistent with its obligation to include subsidence cover; complaint upheld</t>
+        </is>
+      </c>
+      <c r="S33" s="5" t="inlineStr">
+        <is>
+          <t>Insurer arguing that ABI domestic subsidence continuation guidance does not apply because a policy is labelled 'commercial' must look beyond the label to the nature of the building and its occupants — where the building is a residential block effectively owned and occupied by individuals (even through a corporate vehicle), the guidance applies; the good industry practice standard applied by FOS (continue to offer subsidence cover when dealing with a claim) is not limited to the precise terms of the ABI agreement and applies beyond ABI members and beyond purely domestic policies; insurer asserting a policyholder fails its normal underwriting criteria must produce evidence — bare assertion is insufficient; a break in cover caused by a third party's administrative decision does not extinguish the continuation obligation</t>
+        </is>
+      </c>
+      <c r="T33" s="5" t="inlineStr">
+        <is>
+          <t>ABI_continuation_guidance_applies_to_residential_buildings_held_through_corporate_vehicle_where_individual_owners_occupy_as_personal_residence; IF insurer_labels_policy_commercial_BUT_building_is_effectively_residential THEN ABI_continuation_guidance_still_applies; FOS_applies_good_industry_practice_beyond_strict_scope_of_ABI_agreement_and_beyond_ABI_membership; IF insurer_asserts_policyholder_fails_normal_underwriting_criteria THEN insurer_must_produce_evidence_bare_assertion_is_insufficient; break_in_cover_caused_by_third_party_administrative_decision_does_not_extinguish_subsidence_continuation_obligation</t>
+        </is>
+      </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>DRN8561608.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>